<commit_message>
Fases 1 y 2 Propuestas de Roberto
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C234"/>
+  <dimension ref="A1:C245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1075,36 +1075,36 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45853</v>
+        <v>46037</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45854</v>
+        <v>46038</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45856</v>
+        <v>46073</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1114,10 +1114,10 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45857</v>
+        <v>46074</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45884</v>
+        <v>46075</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1143,11 +1143,11 @@
         <v>2</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45887</v>
+        <v>45853</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1156,11 +1156,11 @@
         <v>2</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45888</v>
+        <v>45854</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1169,11 +1169,11 @@
         <v>2</v>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45992</v>
+        <v>45856</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1182,11 +1182,11 @@
         <v>2</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45993</v>
+        <v>45857</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
         <v>2</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45994</v>
+        <v>45884</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1208,11 +1208,11 @@
         <v>2</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45995</v>
+        <v>45887</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1221,11 +1221,11 @@
         <v>2</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45996</v>
+        <v>45888</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1234,11 +1234,11 @@
         <v>2</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
         <v>2</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1260,11 +1260,11 @@
         <v>2</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
         <v>2</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1286,11 +1286,11 @@
         <v>2</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1299,11 +1299,11 @@
         <v>2</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
         <v>2</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
         <v>2</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1338,7 +1338,7 @@
         <v>2</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
         <v>2</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -1364,7 +1364,7 @@
         <v>2</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -1377,11 +1377,11 @@
         <v>2</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1390,11 +1390,11 @@
         <v>2</v>
       </c>
       <c r="B74" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
         <v>2</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -1416,11 +1416,11 @@
         <v>2</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1429,11 +1429,11 @@
         <v>2</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1442,11 +1442,11 @@
         <v>2</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1455,11 +1455,11 @@
         <v>2</v>
       </c>
       <c r="B79" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
         <v>2</v>
       </c>
       <c r="B80" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -1481,11 +1481,11 @@
         <v>2</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1494,11 +1494,11 @@
         <v>2</v>
       </c>
       <c r="B82" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1507,11 +1507,11 @@
         <v>2</v>
       </c>
       <c r="B83" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1520,11 +1520,11 @@
         <v>2</v>
       </c>
       <c r="B84" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1533,11 +1533,11 @@
         <v>2</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1546,11 +1546,11 @@
         <v>2</v>
       </c>
       <c r="B86" s="2" t="n">
-        <v>46021</v>
+        <v>46016</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1559,11 +1559,11 @@
         <v>2</v>
       </c>
       <c r="B87" s="2" t="n">
-        <v>46055</v>
+        <v>46017</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
         <v>2</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>46056</v>
+        <v>46018</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v>2</v>
       </c>
       <c r="B89" s="2" t="n">
-        <v>46057</v>
+        <v>46019</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -1595,10 +1595,10 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B90" s="2" t="n">
-        <v>45850</v>
+        <v>46020</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -1608,49 +1608,49 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B91" s="2" t="n">
-        <v>45851</v>
+        <v>46021</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B92" s="2" t="n">
-        <v>45992</v>
+        <v>46055</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>45993</v>
+        <v>46056</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B94" s="2" t="n">
-        <v>45994</v>
+        <v>46057</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -1663,11 +1663,11 @@
         <v>3</v>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45995</v>
+        <v>45850</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1676,11 +1676,11 @@
         <v>3</v>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45996</v>
+        <v>45851</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1689,11 +1689,11 @@
         <v>3</v>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
         <v>3</v>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -1715,11 +1715,11 @@
         <v>3</v>
       </c>
       <c r="B99" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
         <v>3</v>
       </c>
       <c r="B100" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -1741,11 +1741,11 @@
         <v>3</v>
       </c>
       <c r="B101" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1754,11 +1754,11 @@
         <v>3</v>
       </c>
       <c r="B102" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
         <v>3</v>
       </c>
       <c r="B103" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         <v>3</v>
       </c>
       <c r="B104" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         <v>3</v>
       </c>
       <c r="B105" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -1806,7 +1806,7 @@
         <v>3</v>
       </c>
       <c r="B106" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -1819,7 +1819,7 @@
         <v>3</v>
       </c>
       <c r="B107" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -1832,7 +1832,7 @@
         <v>3</v>
       </c>
       <c r="B108" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
         <v>3</v>
       </c>
       <c r="B109" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
         <v>3</v>
       </c>
       <c r="B110" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -1871,11 +1871,11 @@
         <v>3</v>
       </c>
       <c r="B111" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1884,11 +1884,11 @@
         <v>3</v>
       </c>
       <c r="B112" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
         <v>3</v>
       </c>
       <c r="B113" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -1910,7 +1910,7 @@
         <v>3</v>
       </c>
       <c r="B114" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
         <v>3</v>
       </c>
       <c r="B115" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -1936,11 +1936,11 @@
         <v>3</v>
       </c>
       <c r="B116" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1949,11 +1949,11 @@
         <v>3</v>
       </c>
       <c r="B117" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
         <v>3</v>
       </c>
       <c r="B118" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -1975,7 +1975,7 @@
         <v>3</v>
       </c>
       <c r="B119" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -1988,11 +1988,11 @@
         <v>3</v>
       </c>
       <c r="B120" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2001,20 +2001,20 @@
         <v>3</v>
       </c>
       <c r="B121" s="2" t="n">
-        <v>46021</v>
+        <v>46016</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B122" s="2" t="n">
-        <v>45658</v>
+        <v>46017</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -2024,10 +2024,10 @@
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B123" s="2" t="n">
-        <v>45659</v>
+        <v>46018</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -2037,10 +2037,10 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B124" s="2" t="n">
-        <v>45660</v>
+        <v>46019</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -2050,23 +2050,23 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B125" s="2" t="n">
-        <v>45661</v>
+        <v>46020</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B126" s="2" t="n">
-        <v>45992</v>
+        <v>46021</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>4</v>
       </c>
       <c r="B127" s="2" t="n">
-        <v>45993</v>
+        <v>45658</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -2092,11 +2092,11 @@
         <v>4</v>
       </c>
       <c r="B128" s="2" t="n">
-        <v>45994</v>
+        <v>45659</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
         <v>4</v>
       </c>
       <c r="B129" s="2" t="n">
-        <v>45995</v>
+        <v>45660</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         <v>4</v>
       </c>
       <c r="B130" s="2" t="n">
-        <v>45996</v>
+        <v>45661</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -2131,11 +2131,11 @@
         <v>4</v>
       </c>
       <c r="B131" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
         <v>4</v>
       </c>
       <c r="B132" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
@@ -2157,11 +2157,11 @@
         <v>4</v>
       </c>
       <c r="B133" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
         <v>4</v>
       </c>
       <c r="B134" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
@@ -2183,11 +2183,11 @@
         <v>4</v>
       </c>
       <c r="B135" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2196,11 +2196,11 @@
         <v>4</v>
       </c>
       <c r="B136" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
         <v>4</v>
       </c>
       <c r="B137" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
         <v>4</v>
       </c>
       <c r="B138" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
         <v>4</v>
       </c>
       <c r="B139" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         <v>4</v>
       </c>
       <c r="B140" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         <v>4</v>
       </c>
       <c r="B141" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         <v>4</v>
       </c>
       <c r="B142" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v>4</v>
       </c>
       <c r="B143" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v>4</v>
       </c>
       <c r="B144" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -2313,11 +2313,11 @@
         <v>4</v>
       </c>
       <c r="B145" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2326,11 +2326,11 @@
         <v>4</v>
       </c>
       <c r="B146" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
         <v>4</v>
       </c>
       <c r="B147" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -2352,7 +2352,7 @@
         <v>4</v>
       </c>
       <c r="B148" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         <v>4</v>
       </c>
       <c r="B149" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
@@ -2378,11 +2378,11 @@
         <v>4</v>
       </c>
       <c r="B150" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2391,11 +2391,11 @@
         <v>4</v>
       </c>
       <c r="B151" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
         <v>4</v>
       </c>
       <c r="B152" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
         <v>4</v>
       </c>
       <c r="B153" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
@@ -2430,11 +2430,11 @@
         <v>4</v>
       </c>
       <c r="B154" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2443,11 +2443,11 @@
         <v>4</v>
       </c>
       <c r="B155" s="2" t="n">
-        <v>46021</v>
+        <v>46016</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2456,11 +2456,11 @@
         <v>4</v>
       </c>
       <c r="B156" s="2" t="n">
-        <v>46023</v>
+        <v>46017</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2469,11 +2469,11 @@
         <v>4</v>
       </c>
       <c r="B157" s="2" t="n">
-        <v>46024</v>
+        <v>46018</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2482,11 +2482,11 @@
         <v>4</v>
       </c>
       <c r="B158" s="2" t="n">
-        <v>46025</v>
+        <v>46019</v>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
         <v>4</v>
       </c>
       <c r="B159" s="2" t="n">
-        <v>46026</v>
+        <v>46020</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -2508,11 +2508,11 @@
         <v>4</v>
       </c>
       <c r="B160" s="2" t="n">
-        <v>46027</v>
+        <v>46021</v>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
         <v>4</v>
       </c>
       <c r="B161" s="2" t="n">
-        <v>46028</v>
+        <v>46023</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
@@ -2531,36 +2531,36 @@
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B162" s="2" t="n">
-        <v>45992</v>
+        <v>46024</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B163" s="2" t="n">
-        <v>45993</v>
+        <v>46025</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B164" s="2" t="n">
-        <v>45994</v>
+        <v>46026</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
@@ -2570,49 +2570,49 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B165" s="2" t="n">
-        <v>45995</v>
+        <v>46027</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B166" s="2" t="n">
-        <v>45996</v>
+        <v>46028</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B167" s="2" t="n">
-        <v>45997</v>
+        <v>46038</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B168" s="2" t="n">
-        <v>45998</v>
+        <v>46039</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -2622,10 +2622,10 @@
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B169" s="2" t="n">
-        <v>45999</v>
+        <v>46063</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -2635,10 +2635,10 @@
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B170" s="2" t="n">
-        <v>46000</v>
+        <v>46064</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
@@ -2648,10 +2648,10 @@
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B171" s="2" t="n">
-        <v>46001</v>
+        <v>46078</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
@@ -2661,14 +2661,14 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B172" s="2" t="n">
-        <v>46002</v>
+        <v>46079</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2677,11 +2677,11 @@
         <v>5</v>
       </c>
       <c r="B173" s="2" t="n">
-        <v>46003</v>
+        <v>45992</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2690,11 +2690,11 @@
         <v>5</v>
       </c>
       <c r="B174" s="2" t="n">
-        <v>46004</v>
+        <v>45993</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2703,11 +2703,11 @@
         <v>5</v>
       </c>
       <c r="B175" s="2" t="n">
-        <v>46005</v>
+        <v>45994</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2716,11 +2716,11 @@
         <v>5</v>
       </c>
       <c r="B176" s="2" t="n">
-        <v>46006</v>
+        <v>45995</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>5</v>
       </c>
       <c r="B177" s="2" t="n">
-        <v>46007</v>
+        <v>45996</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
@@ -2742,11 +2742,11 @@
         <v>5</v>
       </c>
       <c r="B178" s="2" t="n">
-        <v>46008</v>
+        <v>45997</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
         <v>5</v>
       </c>
       <c r="B179" s="2" t="n">
-        <v>46009</v>
+        <v>45998</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
@@ -2768,7 +2768,7 @@
         <v>5</v>
       </c>
       <c r="B180" s="2" t="n">
-        <v>46010</v>
+        <v>45999</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
@@ -2781,7 +2781,7 @@
         <v>5</v>
       </c>
       <c r="B181" s="2" t="n">
-        <v>46011</v>
+        <v>46000</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
@@ -2794,7 +2794,7 @@
         <v>5</v>
       </c>
       <c r="B182" s="2" t="n">
-        <v>46012</v>
+        <v>46001</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
         <v>5</v>
       </c>
       <c r="B183" s="2" t="n">
-        <v>46013</v>
+        <v>46002</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -2820,11 +2820,11 @@
         <v>5</v>
       </c>
       <c r="B184" s="2" t="n">
-        <v>46014</v>
+        <v>46003</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2833,11 +2833,11 @@
         <v>5</v>
       </c>
       <c r="B185" s="2" t="n">
-        <v>46015</v>
+        <v>46004</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2846,11 +2846,11 @@
         <v>5</v>
       </c>
       <c r="B186" s="2" t="n">
-        <v>46016</v>
+        <v>46005</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2859,11 +2859,11 @@
         <v>5</v>
       </c>
       <c r="B187" s="2" t="n">
-        <v>46017</v>
+        <v>46006</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
         <v>5</v>
       </c>
       <c r="B188" s="2" t="n">
-        <v>46018</v>
+        <v>46007</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
@@ -2885,7 +2885,7 @@
         <v>5</v>
       </c>
       <c r="B189" s="2" t="n">
-        <v>46019</v>
+        <v>46008</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -2898,11 +2898,11 @@
         <v>5</v>
       </c>
       <c r="B190" s="2" t="n">
-        <v>46020</v>
+        <v>46009</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
         <v>5</v>
       </c>
       <c r="B191" s="2" t="n">
-        <v>46021</v>
+        <v>46010</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -2921,23 +2921,23 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B192" s="2" t="n">
-        <v>45850</v>
+        <v>46011</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B193" s="2" t="n">
-        <v>45851</v>
+        <v>46012</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -2947,49 +2947,49 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B194" s="2" t="n">
-        <v>45860</v>
+        <v>46013</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B195" s="2" t="n">
-        <v>45861</v>
+        <v>46014</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B196" s="2" t="n">
-        <v>45862</v>
+        <v>46015</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B197" s="2" t="n">
-        <v>45863</v>
+        <v>46016</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -2999,10 +2999,10 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B198" s="2" t="n">
-        <v>45867</v>
+        <v>46017</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
@@ -3012,10 +3012,10 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B199" s="2" t="n">
-        <v>45868</v>
+        <v>46018</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
@@ -3025,10 +3025,10 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B200" s="2" t="n">
-        <v>45869</v>
+        <v>46019</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
@@ -3038,27 +3038,27 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B201" s="2" t="n">
-        <v>45870</v>
+        <v>46020</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B202" s="2" t="n">
-        <v>45884</v>
+        <v>46021</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
         <v>6</v>
       </c>
       <c r="B203" s="2" t="n">
-        <v>45885</v>
+        <v>45850</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
@@ -3080,7 +3080,7 @@
         <v>6</v>
       </c>
       <c r="B204" s="2" t="n">
-        <v>45886</v>
+        <v>45851</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
@@ -3093,11 +3093,11 @@
         <v>6</v>
       </c>
       <c r="B205" s="2" t="n">
-        <v>45992</v>
+        <v>45860</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3106,11 +3106,11 @@
         <v>6</v>
       </c>
       <c r="B206" s="2" t="n">
-        <v>45993</v>
+        <v>45861</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
         <v>6</v>
       </c>
       <c r="B207" s="2" t="n">
-        <v>45994</v>
+        <v>45862</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
@@ -3132,11 +3132,11 @@
         <v>6</v>
       </c>
       <c r="B208" s="2" t="n">
-        <v>45995</v>
+        <v>45863</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
         <v>6</v>
       </c>
       <c r="B209" s="2" t="n">
-        <v>45996</v>
+        <v>45867</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -3158,11 +3158,11 @@
         <v>6</v>
       </c>
       <c r="B210" s="2" t="n">
-        <v>45997</v>
+        <v>45868</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
         <v>6</v>
       </c>
       <c r="B211" s="2" t="n">
-        <v>45998</v>
+        <v>45869</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
@@ -3184,7 +3184,7 @@
         <v>6</v>
       </c>
       <c r="B212" s="2" t="n">
-        <v>45999</v>
+        <v>45870</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
@@ -3197,11 +3197,11 @@
         <v>6</v>
       </c>
       <c r="B213" s="2" t="n">
-        <v>46000</v>
+        <v>45884</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
         <v>6</v>
       </c>
       <c r="B214" s="2" t="n">
-        <v>46001</v>
+        <v>45885</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
@@ -3223,11 +3223,11 @@
         <v>6</v>
       </c>
       <c r="B215" s="2" t="n">
-        <v>46002</v>
+        <v>45886</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         <v>6</v>
       </c>
       <c r="B216" s="2" t="n">
-        <v>46003</v>
+        <v>45992</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
@@ -3249,7 +3249,7 @@
         <v>6</v>
       </c>
       <c r="B217" s="2" t="n">
-        <v>46004</v>
+        <v>45993</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
@@ -3262,11 +3262,11 @@
         <v>6</v>
       </c>
       <c r="B218" s="2" t="n">
-        <v>46005</v>
+        <v>45994</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3275,11 +3275,11 @@
         <v>6</v>
       </c>
       <c r="B219" s="2" t="n">
-        <v>46006</v>
+        <v>45995</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3288,7 @@
         <v>6</v>
       </c>
       <c r="B220" s="2" t="n">
-        <v>46007</v>
+        <v>45996</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
@@ -3301,11 +3301,11 @@
         <v>6</v>
       </c>
       <c r="B221" s="2" t="n">
-        <v>46008</v>
+        <v>45997</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
         <v>6</v>
       </c>
       <c r="B222" s="2" t="n">
-        <v>46009</v>
+        <v>45998</v>
       </c>
       <c r="C222" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>6</v>
       </c>
       <c r="B223" s="2" t="n">
-        <v>46010</v>
+        <v>45999</v>
       </c>
       <c r="C223" t="inlineStr">
         <is>
@@ -3340,7 +3340,7 @@
         <v>6</v>
       </c>
       <c r="B224" s="2" t="n">
-        <v>46011</v>
+        <v>46000</v>
       </c>
       <c r="C224" t="inlineStr">
         <is>
@@ -3353,7 +3353,7 @@
         <v>6</v>
       </c>
       <c r="B225" s="2" t="n">
-        <v>46012</v>
+        <v>46001</v>
       </c>
       <c r="C225" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
         <v>6</v>
       </c>
       <c r="B226" s="2" t="n">
-        <v>46013</v>
+        <v>46002</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
@@ -3379,7 +3379,7 @@
         <v>6</v>
       </c>
       <c r="B227" s="2" t="n">
-        <v>46014</v>
+        <v>46003</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
@@ -3392,7 +3392,7 @@
         <v>6</v>
       </c>
       <c r="B228" s="2" t="n">
-        <v>46015</v>
+        <v>46004</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
@@ -3405,11 +3405,11 @@
         <v>6</v>
       </c>
       <c r="B229" s="2" t="n">
-        <v>46016</v>
+        <v>46005</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3418,11 +3418,11 @@
         <v>6</v>
       </c>
       <c r="B230" s="2" t="n">
-        <v>46017</v>
+        <v>46006</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
         <v>6</v>
       </c>
       <c r="B231" s="2" t="n">
-        <v>46018</v>
+        <v>46007</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
@@ -3444,7 +3444,7 @@
         <v>6</v>
       </c>
       <c r="B232" s="2" t="n">
-        <v>46019</v>
+        <v>46008</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
@@ -3457,11 +3457,11 @@
         <v>6</v>
       </c>
       <c r="B233" s="2" t="n">
-        <v>46020</v>
+        <v>46009</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3470,9 +3470,152 @@
         <v>6</v>
       </c>
       <c r="B234" s="2" t="n">
+        <v>46010</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>6</v>
+      </c>
+      <c r="B235" s="2" t="n">
+        <v>46011</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>6</v>
+      </c>
+      <c r="B236" s="2" t="n">
+        <v>46012</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>6</v>
+      </c>
+      <c r="B237" s="2" t="n">
+        <v>46013</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>6</v>
+      </c>
+      <c r="B238" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>6</v>
+      </c>
+      <c r="B239" s="2" t="n">
+        <v>46015</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>6</v>
+      </c>
+      <c r="B240" s="2" t="n">
+        <v>46016</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>6</v>
+      </c>
+      <c r="B241" s="2" t="n">
+        <v>46017</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>6</v>
+      </c>
+      <c r="B242" s="2" t="n">
+        <v>46018</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>6</v>
+      </c>
+      <c r="B243" s="2" t="n">
+        <v>46019</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>6</v>
+      </c>
+      <c r="B244" s="2" t="n">
+        <v>46020</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>6</v>
+      </c>
+      <c r="B245" s="2" t="n">
         <v>46021</v>
       </c>
-      <c r="C234" t="inlineStr">
+      <c r="C245" t="inlineStr">
         <is>
           <t>libre</t>
         </is>

</xml_diff>

<commit_message>
Fase 5 (Admin, chat de admin, tablas, nuevo front)
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cambios Memoria en sucio
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C260"/>
+  <dimension ref="A1:C268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -523,7 +523,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2271,66 +2271,66 @@
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B142" s="2" t="n">
-        <v>45658</v>
+        <v>46392</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B143" s="2" t="n">
-        <v>45659</v>
+        <v>46393</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B144" s="2" t="n">
-        <v>45660</v>
+        <v>46394</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B145" s="2" t="n">
-        <v>45661</v>
+        <v>46395</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B146" s="2" t="n">
-        <v>45992</v>
+        <v>46396</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
         <v>4</v>
       </c>
       <c r="B147" s="2" t="n">
-        <v>45993</v>
+        <v>45658</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -2352,11 +2352,11 @@
         <v>4</v>
       </c>
       <c r="B148" s="2" t="n">
-        <v>45994</v>
+        <v>45659</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
         <v>4</v>
       </c>
       <c r="B149" s="2" t="n">
-        <v>45995</v>
+        <v>45660</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
@@ -2378,7 +2378,7 @@
         <v>4</v>
       </c>
       <c r="B150" s="2" t="n">
-        <v>45996</v>
+        <v>45661</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
@@ -2391,11 +2391,11 @@
         <v>4</v>
       </c>
       <c r="B151" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
         <v>4</v>
       </c>
       <c r="B152" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
@@ -2417,11 +2417,11 @@
         <v>4</v>
       </c>
       <c r="B153" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2430,7 @@
         <v>4</v>
       </c>
       <c r="B154" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -2443,11 +2443,11 @@
         <v>4</v>
       </c>
       <c r="B155" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2456,11 +2456,11 @@
         <v>4</v>
       </c>
       <c r="B156" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
         <v>4</v>
       </c>
       <c r="B157" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         <v>4</v>
       </c>
       <c r="B158" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C158" t="inlineStr">
         <is>
@@ -2495,7 +2495,7 @@
         <v>4</v>
       </c>
       <c r="B159" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -2508,7 +2508,7 @@
         <v>4</v>
       </c>
       <c r="B160" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C160" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         <v>4</v>
       </c>
       <c r="B161" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         <v>4</v>
       </c>
       <c r="B162" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -2547,7 +2547,7 @@
         <v>4</v>
       </c>
       <c r="B163" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         <v>4</v>
       </c>
       <c r="B164" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
@@ -2573,11 +2573,11 @@
         <v>4</v>
       </c>
       <c r="B165" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2586,11 +2586,11 @@
         <v>4</v>
       </c>
       <c r="B166" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
         <v>4</v>
       </c>
       <c r="B167" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
@@ -2612,7 +2612,7 @@
         <v>4</v>
       </c>
       <c r="B168" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
         <v>4</v>
       </c>
       <c r="B169" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -2638,11 +2638,11 @@
         <v>4</v>
       </c>
       <c r="B170" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2651,11 +2651,11 @@
         <v>4</v>
       </c>
       <c r="B171" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
         <v>4</v>
       </c>
       <c r="B172" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         <v>4</v>
       </c>
       <c r="B173" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
@@ -2690,11 +2690,11 @@
         <v>4</v>
       </c>
       <c r="B174" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2703,11 +2703,11 @@
         <v>4</v>
       </c>
       <c r="B175" s="2" t="n">
-        <v>46021</v>
+        <v>46016</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
         <v>4</v>
       </c>
       <c r="B176" s="2" t="n">
-        <v>46023</v>
+        <v>46017</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
@@ -2729,7 +2729,7 @@
         <v>4</v>
       </c>
       <c r="B177" s="2" t="n">
-        <v>46024</v>
+        <v>46018</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
         <v>4</v>
       </c>
       <c r="B178" s="2" t="n">
-        <v>46025</v>
+        <v>46019</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
@@ -2755,11 +2755,11 @@
         <v>4</v>
       </c>
       <c r="B179" s="2" t="n">
-        <v>46026</v>
+        <v>46020</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
         <v>4</v>
       </c>
       <c r="B180" s="2" t="n">
-        <v>46027</v>
+        <v>46021</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
@@ -2781,7 +2781,7 @@
         <v>4</v>
       </c>
       <c r="B181" s="2" t="n">
-        <v>46028</v>
+        <v>46023</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
@@ -2794,7 +2794,7 @@
         <v>4</v>
       </c>
       <c r="B182" s="2" t="n">
-        <v>46038</v>
+        <v>46024</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
         <v>4</v>
       </c>
       <c r="B183" s="2" t="n">
-        <v>46039</v>
+        <v>46025</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
         <v>4</v>
       </c>
       <c r="B184" s="2" t="n">
-        <v>46063</v>
+        <v>46026</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         <v>4</v>
       </c>
       <c r="B185" s="2" t="n">
-        <v>46064</v>
+        <v>46027</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -2846,11 +2846,11 @@
         <v>4</v>
       </c>
       <c r="B186" s="2" t="n">
-        <v>46078</v>
+        <v>46028</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2859,20 +2859,20 @@
         <v>4</v>
       </c>
       <c r="B187" s="2" t="n">
-        <v>46079</v>
+        <v>46038</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B188" s="2" t="n">
-        <v>45992</v>
+        <v>46039</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
@@ -2882,10 +2882,10 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B189" s="2" t="n">
-        <v>45993</v>
+        <v>46042</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -2895,23 +2895,23 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B190" s="2" t="n">
-        <v>45994</v>
+        <v>46043</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B191" s="2" t="n">
-        <v>45995</v>
+        <v>46044</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -2921,10 +2921,10 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B192" s="2" t="n">
-        <v>45996</v>
+        <v>46063</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -2934,40 +2934,40 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B193" s="2" t="n">
-        <v>45997</v>
+        <v>46064</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B194" s="2" t="n">
-        <v>45998</v>
+        <v>46078</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B195" s="2" t="n">
-        <v>45999</v>
+        <v>46079</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
         <v>5</v>
       </c>
       <c r="B196" s="2" t="n">
-        <v>46000</v>
+        <v>45992</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -2989,11 +2989,11 @@
         <v>5</v>
       </c>
       <c r="B197" s="2" t="n">
-        <v>46001</v>
+        <v>45993</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3002,11 +3002,11 @@
         <v>5</v>
       </c>
       <c r="B198" s="2" t="n">
-        <v>46002</v>
+        <v>45994</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3015,11 +3015,11 @@
         <v>5</v>
       </c>
       <c r="B199" s="2" t="n">
-        <v>46003</v>
+        <v>45995</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3028,11 +3028,11 @@
         <v>5</v>
       </c>
       <c r="B200" s="2" t="n">
-        <v>46004</v>
+        <v>45996</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3041,11 +3041,11 @@
         <v>5</v>
       </c>
       <c r="B201" s="2" t="n">
-        <v>46005</v>
+        <v>45997</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3054,11 +3054,11 @@
         <v>5</v>
       </c>
       <c r="B202" s="2" t="n">
-        <v>46006</v>
+        <v>45998</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
         <v>5</v>
       </c>
       <c r="B203" s="2" t="n">
-        <v>46007</v>
+        <v>45999</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
@@ -3080,7 +3080,7 @@
         <v>5</v>
       </c>
       <c r="B204" s="2" t="n">
-        <v>46008</v>
+        <v>46000</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
@@ -3093,11 +3093,11 @@
         <v>5</v>
       </c>
       <c r="B205" s="2" t="n">
-        <v>46009</v>
+        <v>46001</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3106,7 @@
         <v>5</v>
       </c>
       <c r="B206" s="2" t="n">
-        <v>46010</v>
+        <v>46002</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
@@ -3119,11 +3119,11 @@
         <v>5</v>
       </c>
       <c r="B207" s="2" t="n">
-        <v>46011</v>
+        <v>46003</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3132,7 +3132,7 @@
         <v>5</v>
       </c>
       <c r="B208" s="2" t="n">
-        <v>46012</v>
+        <v>46004</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
@@ -3145,7 +3145,7 @@
         <v>5</v>
       </c>
       <c r="B209" s="2" t="n">
-        <v>46013</v>
+        <v>46005</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -3158,11 +3158,11 @@
         <v>5</v>
       </c>
       <c r="B210" s="2" t="n">
-        <v>46014</v>
+        <v>46006</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
         <v>5</v>
       </c>
       <c r="B211" s="2" t="n">
-        <v>46015</v>
+        <v>46007</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
@@ -3184,11 +3184,11 @@
         <v>5</v>
       </c>
       <c r="B212" s="2" t="n">
-        <v>46016</v>
+        <v>46008</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         <v>5</v>
       </c>
       <c r="B213" s="2" t="n">
-        <v>46017</v>
+        <v>46009</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
@@ -3210,7 +3210,7 @@
         <v>5</v>
       </c>
       <c r="B214" s="2" t="n">
-        <v>46018</v>
+        <v>46010</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
         <v>5</v>
       </c>
       <c r="B215" s="2" t="n">
-        <v>46019</v>
+        <v>46011</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         <v>5</v>
       </c>
       <c r="B216" s="2" t="n">
-        <v>46020</v>
+        <v>46012</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
@@ -3249,7 +3249,7 @@
         <v>5</v>
       </c>
       <c r="B217" s="2" t="n">
-        <v>46021</v>
+        <v>46013</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
@@ -3259,36 +3259,36 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B218" s="2" t="n">
-        <v>45850</v>
+        <v>46014</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B219" s="2" t="n">
-        <v>45851</v>
+        <v>46015</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B220" s="2" t="n">
-        <v>45860</v>
+        <v>46016</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
@@ -3298,62 +3298,62 @@
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B221" s="2" t="n">
-        <v>45861</v>
+        <v>46017</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B222" s="2" t="n">
-        <v>45862</v>
+        <v>46018</v>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B223" s="2" t="n">
-        <v>45863</v>
+        <v>46019</v>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B224" s="2" t="n">
-        <v>45867</v>
+        <v>46020</v>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B225" s="2" t="n">
-        <v>45868</v>
+        <v>46021</v>
       </c>
       <c r="C225" t="inlineStr">
         <is>
@@ -3366,11 +3366,11 @@
         <v>6</v>
       </c>
       <c r="B226" s="2" t="n">
-        <v>45869</v>
+        <v>45850</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3379,11 +3379,11 @@
         <v>6</v>
       </c>
       <c r="B227" s="2" t="n">
-        <v>45870</v>
+        <v>45851</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
         <v>6</v>
       </c>
       <c r="B228" s="2" t="n">
-        <v>45884</v>
+        <v>45860</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
@@ -3405,7 +3405,7 @@
         <v>6</v>
       </c>
       <c r="B229" s="2" t="n">
-        <v>45885</v>
+        <v>45861</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
@@ -3418,7 +3418,7 @@
         <v>6</v>
       </c>
       <c r="B230" s="2" t="n">
-        <v>45886</v>
+        <v>45862</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
@@ -3431,11 +3431,11 @@
         <v>6</v>
       </c>
       <c r="B231" s="2" t="n">
-        <v>45992</v>
+        <v>45863</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3444,7 @@
         <v>6</v>
       </c>
       <c r="B232" s="2" t="n">
-        <v>45993</v>
+        <v>45867</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
@@ -3457,11 +3457,11 @@
         <v>6</v>
       </c>
       <c r="B233" s="2" t="n">
-        <v>45994</v>
+        <v>45868</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
         <v>6</v>
       </c>
       <c r="B234" s="2" t="n">
-        <v>45995</v>
+        <v>45869</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>6</v>
       </c>
       <c r="B235" s="2" t="n">
-        <v>45996</v>
+        <v>45870</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
@@ -3496,7 +3496,7 @@
         <v>6</v>
       </c>
       <c r="B236" s="2" t="n">
-        <v>45997</v>
+        <v>45884</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -3509,11 +3509,11 @@
         <v>6</v>
       </c>
       <c r="B237" s="2" t="n">
-        <v>45998</v>
+        <v>45885</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3522,11 +3522,11 @@
         <v>6</v>
       </c>
       <c r="B238" s="2" t="n">
-        <v>45999</v>
+        <v>45886</v>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
         <v>6</v>
       </c>
       <c r="B239" s="2" t="n">
-        <v>46000</v>
+        <v>45992</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -3548,11 +3548,11 @@
         <v>6</v>
       </c>
       <c r="B240" s="2" t="n">
-        <v>46001</v>
+        <v>45993</v>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3561,11 +3561,11 @@
         <v>6</v>
       </c>
       <c r="B241" s="2" t="n">
-        <v>46002</v>
+        <v>45994</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
         <v>6</v>
       </c>
       <c r="B242" s="2" t="n">
-        <v>46003</v>
+        <v>45995</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
@@ -3587,7 +3587,7 @@
         <v>6</v>
       </c>
       <c r="B243" s="2" t="n">
-        <v>46004</v>
+        <v>45996</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
@@ -3600,11 +3600,11 @@
         <v>6</v>
       </c>
       <c r="B244" s="2" t="n">
-        <v>46005</v>
+        <v>45997</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3613,11 +3613,11 @@
         <v>6</v>
       </c>
       <c r="B245" s="2" t="n">
-        <v>46006</v>
+        <v>45998</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
         <v>6</v>
       </c>
       <c r="B246" s="2" t="n">
-        <v>46007</v>
+        <v>45999</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
@@ -3639,7 +3639,7 @@
         <v>6</v>
       </c>
       <c r="B247" s="2" t="n">
-        <v>46008</v>
+        <v>46000</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -3652,11 +3652,11 @@
         <v>6</v>
       </c>
       <c r="B248" s="2" t="n">
-        <v>46009</v>
+        <v>46001</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="n">
-        <v>46010</v>
+        <v>46002</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         <v>6</v>
       </c>
       <c r="B250" s="2" t="n">
-        <v>46011</v>
+        <v>46003</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -3691,11 +3691,11 @@
         <v>6</v>
       </c>
       <c r="B251" s="2" t="n">
-        <v>46012</v>
+        <v>46004</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3704,7 @@
         <v>6</v>
       </c>
       <c r="B252" s="2" t="n">
-        <v>46013</v>
+        <v>46005</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -3717,11 +3717,11 @@
         <v>6</v>
       </c>
       <c r="B253" s="2" t="n">
-        <v>46014</v>
+        <v>46006</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3730,7 +3730,7 @@
         <v>6</v>
       </c>
       <c r="B254" s="2" t="n">
-        <v>46015</v>
+        <v>46007</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
@@ -3743,11 +3743,11 @@
         <v>6</v>
       </c>
       <c r="B255" s="2" t="n">
-        <v>46016</v>
+        <v>46008</v>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3756,7 +3756,7 @@
         <v>6</v>
       </c>
       <c r="B256" s="2" t="n">
-        <v>46017</v>
+        <v>46009</v>
       </c>
       <c r="C256" t="inlineStr">
         <is>
@@ -3769,7 +3769,7 @@
         <v>6</v>
       </c>
       <c r="B257" s="2" t="n">
-        <v>46018</v>
+        <v>46010</v>
       </c>
       <c r="C257" t="inlineStr">
         <is>
@@ -3782,7 +3782,7 @@
         <v>6</v>
       </c>
       <c r="B258" s="2" t="n">
-        <v>46019</v>
+        <v>46011</v>
       </c>
       <c r="C258" t="inlineStr">
         <is>
@@ -3795,7 +3795,7 @@
         <v>6</v>
       </c>
       <c r="B259" s="2" t="n">
-        <v>46020</v>
+        <v>46012</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
@@ -3808,9 +3808,113 @@
         <v>6</v>
       </c>
       <c r="B260" s="2" t="n">
+        <v>46013</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>6</v>
+      </c>
+      <c r="B261" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>6</v>
+      </c>
+      <c r="B262" s="2" t="n">
+        <v>46015</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>6</v>
+      </c>
+      <c r="B263" s="2" t="n">
+        <v>46016</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>6</v>
+      </c>
+      <c r="B264" s="2" t="n">
+        <v>46017</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>6</v>
+      </c>
+      <c r="B265" s="2" t="n">
+        <v>46018</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>6</v>
+      </c>
+      <c r="B266" s="2" t="n">
+        <v>46019</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>6</v>
+      </c>
+      <c r="B267" s="2" t="n">
+        <v>46020</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>6</v>
+      </c>
+      <c r="B268" s="2" t="n">
         <v>46021</v>
       </c>
-      <c r="C260" t="inlineStr">
+      <c r="C268" t="inlineStr">
         <is>
           <t>libre</t>
         </is>

</xml_diff>

<commit_message>
indice memoria y modificaciones
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C268"/>
+  <dimension ref="A1:C273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1140,36 +1140,36 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45853</v>
+        <v>46076</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45854</v>
+        <v>46077</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45856</v>
+        <v>46078</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1182,11 +1182,11 @@
         <v>2</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45857</v>
+        <v>45853</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1195,11 +1195,11 @@
         <v>2</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45884</v>
+        <v>45854</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
         <v>2</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45887</v>
+        <v>45856</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         <v>2</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45888</v>
+        <v>45857</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1234,11 +1234,11 @@
         <v>2</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45992</v>
+        <v>45884</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1247,11 +1247,11 @@
         <v>2</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45993</v>
+        <v>45887</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
         <v>2</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45994</v>
+        <v>45888</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         <v>2</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45995</v>
+        <v>45992</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1286,7 +1286,7 @@
         <v>2</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45996</v>
+        <v>45993</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         <v>2</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45997</v>
+        <v>45994</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         <v>2</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45998</v>
+        <v>45995</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
         <v>2</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45999</v>
+        <v>45996</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1338,11 +1338,11 @@
         <v>2</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>46000</v>
+        <v>45997</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1351,11 +1351,11 @@
         <v>2</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>46001</v>
+        <v>45998</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
         <v>2</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>46002</v>
+        <v>45999</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -1377,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>46003</v>
+        <v>46000</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -1390,11 +1390,11 @@
         <v>2</v>
       </c>
       <c r="B74" s="2" t="n">
-        <v>46004</v>
+        <v>46001</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
         <v>2</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>46005</v>
+        <v>46002</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -1416,11 +1416,11 @@
         <v>2</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>46006</v>
+        <v>46003</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
         <v>2</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>46007</v>
+        <v>46004</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -1442,11 +1442,11 @@
         <v>2</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>46008</v>
+        <v>46005</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
         <v>2</v>
       </c>
       <c r="B79" s="2" t="n">
-        <v>46009</v>
+        <v>46006</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         <v>2</v>
       </c>
       <c r="B80" s="2" t="n">
-        <v>46010</v>
+        <v>46007</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -1481,11 +1481,11 @@
         <v>2</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>46011</v>
+        <v>46008</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
         <v>2</v>
       </c>
       <c r="B82" s="2" t="n">
-        <v>46012</v>
+        <v>46009</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
         <v>2</v>
       </c>
       <c r="B83" s="2" t="n">
-        <v>46013</v>
+        <v>46010</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -1520,7 +1520,7 @@
         <v>2</v>
       </c>
       <c r="B84" s="2" t="n">
-        <v>46014</v>
+        <v>46011</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -1533,11 +1533,11 @@
         <v>2</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>46015</v>
+        <v>46012</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1546,11 +1546,11 @@
         <v>2</v>
       </c>
       <c r="B86" s="2" t="n">
-        <v>46016</v>
+        <v>46013</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
         <v>2</v>
       </c>
       <c r="B87" s="2" t="n">
-        <v>46017</v>
+        <v>46014</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -1572,11 +1572,11 @@
         <v>2</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>46018</v>
+        <v>46015</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
         <v>2</v>
       </c>
       <c r="B89" s="2" t="n">
-        <v>46019</v>
+        <v>46016</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -1598,11 +1598,11 @@
         <v>2</v>
       </c>
       <c r="B90" s="2" t="n">
-        <v>46020</v>
+        <v>46017</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1611,11 +1611,11 @@
         <v>2</v>
       </c>
       <c r="B91" s="2" t="n">
-        <v>46021</v>
+        <v>46018</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
         <v>2</v>
       </c>
       <c r="B92" s="2" t="n">
-        <v>46055</v>
+        <v>46019</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -1637,7 +1637,7 @@
         <v>2</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>46056</v>
+        <v>46020</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -1650,20 +1650,20 @@
         <v>2</v>
       </c>
       <c r="B94" s="2" t="n">
-        <v>46057</v>
+        <v>46021</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45850</v>
+        <v>46055</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -1673,10 +1673,10 @@
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45851</v>
+        <v>46056</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -1686,14 +1686,14 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45992</v>
+        <v>46057</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1702,11 +1702,11 @@
         <v>3</v>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45993</v>
+        <v>45850</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
         <v>3</v>
       </c>
       <c r="B99" s="2" t="n">
-        <v>45994</v>
+        <v>45851</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -1728,7 +1728,7 @@
         <v>3</v>
       </c>
       <c r="B100" s="2" t="n">
-        <v>45995</v>
+        <v>45992</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         <v>3</v>
       </c>
       <c r="B101" s="2" t="n">
-        <v>45996</v>
+        <v>45993</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
         <v>3</v>
       </c>
       <c r="B102" s="2" t="n">
-        <v>45997</v>
+        <v>45994</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         <v>3</v>
       </c>
       <c r="B103" s="2" t="n">
-        <v>45998</v>
+        <v>45995</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         <v>3</v>
       </c>
       <c r="B104" s="2" t="n">
-        <v>45999</v>
+        <v>45996</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -1793,11 +1793,11 @@
         <v>3</v>
       </c>
       <c r="B105" s="2" t="n">
-        <v>46000</v>
+        <v>45997</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1806,11 +1806,11 @@
         <v>3</v>
       </c>
       <c r="B106" s="2" t="n">
-        <v>46001</v>
+        <v>45998</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1819,7 @@
         <v>3</v>
       </c>
       <c r="B107" s="2" t="n">
-        <v>46002</v>
+        <v>45999</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -1832,7 +1832,7 @@
         <v>3</v>
       </c>
       <c r="B108" s="2" t="n">
-        <v>46003</v>
+        <v>46000</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -1845,11 +1845,11 @@
         <v>3</v>
       </c>
       <c r="B109" s="2" t="n">
-        <v>46004</v>
+        <v>46001</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
         <v>3</v>
       </c>
       <c r="B110" s="2" t="n">
-        <v>46005</v>
+        <v>46002</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -1871,11 +1871,11 @@
         <v>3</v>
       </c>
       <c r="B111" s="2" t="n">
-        <v>46006</v>
+        <v>46003</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
         <v>3</v>
       </c>
       <c r="B112" s="2" t="n">
-        <v>46007</v>
+        <v>46004</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>3</v>
       </c>
       <c r="B113" s="2" t="n">
-        <v>46008</v>
+        <v>46005</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -1910,11 +1910,11 @@
         <v>3</v>
       </c>
       <c r="B114" s="2" t="n">
-        <v>46009</v>
+        <v>46006</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
         <v>3</v>
       </c>
       <c r="B115" s="2" t="n">
-        <v>46010</v>
+        <v>46007</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -1936,7 +1936,7 @@
         <v>3</v>
       </c>
       <c r="B116" s="2" t="n">
-        <v>46011</v>
+        <v>46008</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -1949,11 +1949,11 @@
         <v>3</v>
       </c>
       <c r="B117" s="2" t="n">
-        <v>46012</v>
+        <v>46009</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
         <v>3</v>
       </c>
       <c r="B118" s="2" t="n">
-        <v>46013</v>
+        <v>46010</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -1975,7 +1975,7 @@
         <v>3</v>
       </c>
       <c r="B119" s="2" t="n">
-        <v>46014</v>
+        <v>46011</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -1988,11 +1988,11 @@
         <v>3</v>
       </c>
       <c r="B120" s="2" t="n">
-        <v>46015</v>
+        <v>46012</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2001,11 +2001,11 @@
         <v>3</v>
       </c>
       <c r="B121" s="2" t="n">
-        <v>46016</v>
+        <v>46013</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
         <v>3</v>
       </c>
       <c r="B122" s="2" t="n">
-        <v>46017</v>
+        <v>46014</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         <v>3</v>
       </c>
       <c r="B123" s="2" t="n">
-        <v>46018</v>
+        <v>46015</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -2040,11 +2040,11 @@
         <v>3</v>
       </c>
       <c r="B124" s="2" t="n">
-        <v>46019</v>
+        <v>46016</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2053,11 +2053,11 @@
         <v>3</v>
       </c>
       <c r="B125" s="2" t="n">
-        <v>46020</v>
+        <v>46017</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
         <v>3</v>
       </c>
       <c r="B126" s="2" t="n">
-        <v>46021</v>
+        <v>46018</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>3</v>
       </c>
       <c r="B127" s="2" t="n">
-        <v>46068</v>
+        <v>46019</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -2092,11 +2092,11 @@
         <v>3</v>
       </c>
       <c r="B128" s="2" t="n">
-        <v>46069</v>
+        <v>46020</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
         <v>3</v>
       </c>
       <c r="B129" s="2" t="n">
-        <v>46070</v>
+        <v>46021</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         <v>3</v>
       </c>
       <c r="B130" s="2" t="n">
-        <v>46071</v>
+        <v>46068</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -2131,11 +2131,11 @@
         <v>3</v>
       </c>
       <c r="B131" s="2" t="n">
-        <v>46073</v>
+        <v>46069</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2144,11 +2144,11 @@
         <v>3</v>
       </c>
       <c r="B132" s="2" t="n">
-        <v>46074</v>
+        <v>46070</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2157,11 +2157,11 @@
         <v>3</v>
       </c>
       <c r="B133" s="2" t="n">
-        <v>46075</v>
+        <v>46071</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
         <v>3</v>
       </c>
       <c r="B134" s="2" t="n">
-        <v>46077</v>
+        <v>46073</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
         <v>3</v>
       </c>
       <c r="B135" s="2" t="n">
-        <v>46078</v>
+        <v>46074</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
@@ -2196,7 +2196,7 @@
         <v>3</v>
       </c>
       <c r="B136" s="2" t="n">
-        <v>46103</v>
+        <v>46075</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
         <v>3</v>
       </c>
       <c r="B137" s="2" t="n">
-        <v>46104</v>
+        <v>46077</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
         <v>3</v>
       </c>
       <c r="B138" s="2" t="n">
-        <v>46105</v>
+        <v>46078</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
         <v>3</v>
       </c>
       <c r="B139" s="2" t="n">
-        <v>46106</v>
+        <v>46079</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         <v>3</v>
       </c>
       <c r="B140" s="2" t="n">
-        <v>46108</v>
+        <v>46080</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         <v>3</v>
       </c>
       <c r="B141" s="2" t="n">
-        <v>46109</v>
+        <v>46103</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         <v>3</v>
       </c>
       <c r="B142" s="2" t="n">
-        <v>46392</v>
+        <v>46104</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v>3</v>
       </c>
       <c r="B143" s="2" t="n">
-        <v>46393</v>
+        <v>46105</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v>3</v>
       </c>
       <c r="B144" s="2" t="n">
-        <v>46394</v>
+        <v>46106</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         <v>3</v>
       </c>
       <c r="B145" s="2" t="n">
-        <v>46395</v>
+        <v>46108</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         <v>3</v>
       </c>
       <c r="B146" s="2" t="n">
-        <v>46396</v>
+        <v>46109</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
@@ -2336,66 +2336,66 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B147" s="2" t="n">
-        <v>45658</v>
+        <v>46392</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B148" s="2" t="n">
-        <v>45659</v>
+        <v>46393</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B149" s="2" t="n">
-        <v>45660</v>
+        <v>46394</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B150" s="2" t="n">
-        <v>45661</v>
+        <v>46395</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B151" s="2" t="n">
-        <v>45992</v>
+        <v>46396</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
         <v>4</v>
       </c>
       <c r="B152" s="2" t="n">
-        <v>45993</v>
+        <v>45658</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
@@ -2417,11 +2417,11 @@
         <v>4</v>
       </c>
       <c r="B153" s="2" t="n">
-        <v>45994</v>
+        <v>45659</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2430,7 @@
         <v>4</v>
       </c>
       <c r="B154" s="2" t="n">
-        <v>45995</v>
+        <v>45660</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
         <v>4</v>
       </c>
       <c r="B155" s="2" t="n">
-        <v>45996</v>
+        <v>45661</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -2456,11 +2456,11 @@
         <v>4</v>
       </c>
       <c r="B156" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
         <v>4</v>
       </c>
       <c r="B157" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
@@ -2482,11 +2482,11 @@
         <v>4</v>
       </c>
       <c r="B158" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
         <v>4</v>
       </c>
       <c r="B159" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -2508,11 +2508,11 @@
         <v>4</v>
       </c>
       <c r="B160" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2521,11 +2521,11 @@
         <v>4</v>
       </c>
       <c r="B161" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
         <v>4</v>
       </c>
       <c r="B162" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -2547,7 +2547,7 @@
         <v>4</v>
       </c>
       <c r="B163" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
@@ -2560,7 +2560,7 @@
         <v>4</v>
       </c>
       <c r="B164" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
         <v>4</v>
       </c>
       <c r="B165" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
         <v>4</v>
       </c>
       <c r="B166" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -2599,7 +2599,7 @@
         <v>4</v>
       </c>
       <c r="B167" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
@@ -2612,7 +2612,7 @@
         <v>4</v>
       </c>
       <c r="B168" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
         <v>4</v>
       </c>
       <c r="B169" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -2638,11 +2638,11 @@
         <v>4</v>
       </c>
       <c r="B170" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2651,11 +2651,11 @@
         <v>4</v>
       </c>
       <c r="B171" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
         <v>4</v>
       </c>
       <c r="B172" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         <v>4</v>
       </c>
       <c r="B173" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
@@ -2690,7 +2690,7 @@
         <v>4</v>
       </c>
       <c r="B174" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
@@ -2703,11 +2703,11 @@
         <v>4</v>
       </c>
       <c r="B175" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2716,11 +2716,11 @@
         <v>4</v>
       </c>
       <c r="B176" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>4</v>
       </c>
       <c r="B177" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
         <v>4</v>
       </c>
       <c r="B178" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
@@ -2755,11 +2755,11 @@
         <v>4</v>
       </c>
       <c r="B179" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2768,11 +2768,11 @@
         <v>4</v>
       </c>
       <c r="B180" s="2" t="n">
-        <v>46021</v>
+        <v>46016</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
         <v>4</v>
       </c>
       <c r="B181" s="2" t="n">
-        <v>46023</v>
+        <v>46017</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
@@ -2794,7 +2794,7 @@
         <v>4</v>
       </c>
       <c r="B182" s="2" t="n">
-        <v>46024</v>
+        <v>46018</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
         <v>4</v>
       </c>
       <c r="B183" s="2" t="n">
-        <v>46025</v>
+        <v>46019</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -2820,11 +2820,11 @@
         <v>4</v>
       </c>
       <c r="B184" s="2" t="n">
-        <v>46026</v>
+        <v>46020</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
         <v>4</v>
       </c>
       <c r="B185" s="2" t="n">
-        <v>46027</v>
+        <v>46021</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -2846,7 +2846,7 @@
         <v>4</v>
       </c>
       <c r="B186" s="2" t="n">
-        <v>46028</v>
+        <v>46023</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
@@ -2859,7 +2859,7 @@
         <v>4</v>
       </c>
       <c r="B187" s="2" t="n">
-        <v>46038</v>
+        <v>46024</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
         <v>4</v>
       </c>
       <c r="B188" s="2" t="n">
-        <v>46039</v>
+        <v>46025</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
@@ -2885,7 +2885,7 @@
         <v>4</v>
       </c>
       <c r="B189" s="2" t="n">
-        <v>46042</v>
+        <v>46026</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
         <v>4</v>
       </c>
       <c r="B190" s="2" t="n">
-        <v>46043</v>
+        <v>46027</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -2911,7 +2911,7 @@
         <v>4</v>
       </c>
       <c r="B191" s="2" t="n">
-        <v>46044</v>
+        <v>46028</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -2924,7 +2924,7 @@
         <v>4</v>
       </c>
       <c r="B192" s="2" t="n">
-        <v>46063</v>
+        <v>46038</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
         <v>4</v>
       </c>
       <c r="B193" s="2" t="n">
-        <v>46064</v>
+        <v>46039</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -2950,11 +2950,11 @@
         <v>4</v>
       </c>
       <c r="B194" s="2" t="n">
-        <v>46078</v>
+        <v>46042</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2963,20 +2963,20 @@
         <v>4</v>
       </c>
       <c r="B195" s="2" t="n">
-        <v>46079</v>
+        <v>46043</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B196" s="2" t="n">
-        <v>45992</v>
+        <v>46044</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -2986,10 +2986,10 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B197" s="2" t="n">
-        <v>45993</v>
+        <v>46063</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -2999,40 +2999,40 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B198" s="2" t="n">
-        <v>45994</v>
+        <v>46064</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B199" s="2" t="n">
-        <v>45995</v>
+        <v>46078</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B200" s="2" t="n">
-        <v>45996</v>
+        <v>46079</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3041,11 +3041,11 @@
         <v>5</v>
       </c>
       <c r="B201" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
         <v>5</v>
       </c>
       <c r="B202" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
@@ -3067,11 +3067,11 @@
         <v>5</v>
       </c>
       <c r="B203" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
         <v>5</v>
       </c>
       <c r="B204" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
@@ -3093,11 +3093,11 @@
         <v>5</v>
       </c>
       <c r="B205" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3106,11 +3106,11 @@
         <v>5</v>
       </c>
       <c r="B206" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3119,11 +3119,11 @@
         <v>5</v>
       </c>
       <c r="B207" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3132,11 +3132,11 @@
         <v>5</v>
       </c>
       <c r="B208" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
         <v>5</v>
       </c>
       <c r="B209" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         <v>5</v>
       </c>
       <c r="B210" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
@@ -3171,7 +3171,7 @@
         <v>5</v>
       </c>
       <c r="B211" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
@@ -3184,11 +3184,11 @@
         <v>5</v>
       </c>
       <c r="B212" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3197,11 +3197,11 @@
         <v>5</v>
       </c>
       <c r="B213" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
         <v>5</v>
       </c>
       <c r="B214" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
@@ -3223,11 +3223,11 @@
         <v>5</v>
       </c>
       <c r="B215" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3236,11 +3236,11 @@
         <v>5</v>
       </c>
       <c r="B216" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3249,7 @@
         <v>5</v>
       </c>
       <c r="B217" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
@@ -3262,7 +3262,7 @@
         <v>5</v>
       </c>
       <c r="B218" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
         <v>5</v>
       </c>
       <c r="B219" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
@@ -3288,11 +3288,11 @@
         <v>5</v>
       </c>
       <c r="B220" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3301,11 +3301,11 @@
         <v>5</v>
       </c>
       <c r="B221" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
         <v>5</v>
       </c>
       <c r="B222" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C222" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>5</v>
       </c>
       <c r="B223" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C223" t="inlineStr">
         <is>
@@ -3340,11 +3340,11 @@
         <v>5</v>
       </c>
       <c r="B224" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3353,59 +3353,59 @@
         <v>5</v>
       </c>
       <c r="B225" s="2" t="n">
-        <v>46021</v>
+        <v>46016</v>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B226" s="2" t="n">
-        <v>45850</v>
+        <v>46017</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B227" s="2" t="n">
-        <v>45851</v>
+        <v>46018</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B228" s="2" t="n">
-        <v>45860</v>
+        <v>46019</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B229" s="2" t="n">
-        <v>45861</v>
+        <v>46020</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
@@ -3415,14 +3415,14 @@
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B230" s="2" t="n">
-        <v>45862</v>
+        <v>46021</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
         <v>6</v>
       </c>
       <c r="B231" s="2" t="n">
-        <v>45863</v>
+        <v>45850</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
@@ -3444,11 +3444,11 @@
         <v>6</v>
       </c>
       <c r="B232" s="2" t="n">
-        <v>45867</v>
+        <v>45851</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3457,11 +3457,11 @@
         <v>6</v>
       </c>
       <c r="B233" s="2" t="n">
-        <v>45868</v>
+        <v>45860</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3470,11 +3470,11 @@
         <v>6</v>
       </c>
       <c r="B234" s="2" t="n">
-        <v>45869</v>
+        <v>45861</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3483,11 +3483,11 @@
         <v>6</v>
       </c>
       <c r="B235" s="2" t="n">
-        <v>45870</v>
+        <v>45862</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>6</v>
       </c>
       <c r="B236" s="2" t="n">
-        <v>45884</v>
+        <v>45863</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -3509,11 +3509,11 @@
         <v>6</v>
       </c>
       <c r="B237" s="2" t="n">
-        <v>45885</v>
+        <v>45867</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3522,11 +3522,11 @@
         <v>6</v>
       </c>
       <c r="B238" s="2" t="n">
-        <v>45886</v>
+        <v>45868</v>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
         <v>6</v>
       </c>
       <c r="B239" s="2" t="n">
-        <v>45992</v>
+        <v>45869</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
         <v>6</v>
       </c>
       <c r="B240" s="2" t="n">
-        <v>45993</v>
+        <v>45870</v>
       </c>
       <c r="C240" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
         <v>6</v>
       </c>
       <c r="B241" s="2" t="n">
-        <v>45994</v>
+        <v>45884</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
@@ -3574,11 +3574,11 @@
         <v>6</v>
       </c>
       <c r="B242" s="2" t="n">
-        <v>45995</v>
+        <v>45885</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3587,11 +3587,11 @@
         <v>6</v>
       </c>
       <c r="B243" s="2" t="n">
-        <v>45996</v>
+        <v>45886</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3600,11 +3600,11 @@
         <v>6</v>
       </c>
       <c r="B244" s="2" t="n">
-        <v>45997</v>
+        <v>45992</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
         <v>6</v>
       </c>
       <c r="B245" s="2" t="n">
-        <v>45998</v>
+        <v>45993</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
@@ -3626,11 +3626,11 @@
         <v>6</v>
       </c>
       <c r="B246" s="2" t="n">
-        <v>45999</v>
+        <v>45994</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
         <v>6</v>
       </c>
       <c r="B247" s="2" t="n">
-        <v>46000</v>
+        <v>45995</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -3652,11 +3652,11 @@
         <v>6</v>
       </c>
       <c r="B248" s="2" t="n">
-        <v>46001</v>
+        <v>45996</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3665,11 +3665,11 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3678,7 @@
         <v>6</v>
       </c>
       <c r="B250" s="2" t="n">
-        <v>46003</v>
+        <v>45998</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
         <v>6</v>
       </c>
       <c r="B251" s="2" t="n">
-        <v>46004</v>
+        <v>45999</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
         <v>6</v>
       </c>
       <c r="B252" s="2" t="n">
-        <v>46005</v>
+        <v>46000</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -3717,7 +3717,7 @@
         <v>6</v>
       </c>
       <c r="B253" s="2" t="n">
-        <v>46006</v>
+        <v>46001</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
@@ -3730,7 +3730,7 @@
         <v>6</v>
       </c>
       <c r="B254" s="2" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
@@ -3743,7 +3743,7 @@
         <v>6</v>
       </c>
       <c r="B255" s="2" t="n">
-        <v>46008</v>
+        <v>46003</v>
       </c>
       <c r="C255" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         <v>6</v>
       </c>
       <c r="B256" s="2" t="n">
-        <v>46009</v>
+        <v>46004</v>
       </c>
       <c r="C256" t="inlineStr">
         <is>
@@ -3769,7 +3769,7 @@
         <v>6</v>
       </c>
       <c r="B257" s="2" t="n">
-        <v>46010</v>
+        <v>46005</v>
       </c>
       <c r="C257" t="inlineStr">
         <is>
@@ -3782,11 +3782,11 @@
         <v>6</v>
       </c>
       <c r="B258" s="2" t="n">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3795,11 +3795,11 @@
         <v>6</v>
       </c>
       <c r="B259" s="2" t="n">
-        <v>46012</v>
+        <v>46007</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
         <v>6</v>
       </c>
       <c r="B260" s="2" t="n">
-        <v>46013</v>
+        <v>46008</v>
       </c>
       <c r="C260" t="inlineStr">
         <is>
@@ -3821,7 +3821,7 @@
         <v>6</v>
       </c>
       <c r="B261" s="2" t="n">
-        <v>46014</v>
+        <v>46009</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
@@ -3834,7 +3834,7 @@
         <v>6</v>
       </c>
       <c r="B262" s="2" t="n">
-        <v>46015</v>
+        <v>46010</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
@@ -3847,11 +3847,11 @@
         <v>6</v>
       </c>
       <c r="B263" s="2" t="n">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3860,11 +3860,11 @@
         <v>6</v>
       </c>
       <c r="B264" s="2" t="n">
-        <v>46017</v>
+        <v>46012</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3873,7 +3873,7 @@
         <v>6</v>
       </c>
       <c r="B265" s="2" t="n">
-        <v>46018</v>
+        <v>46013</v>
       </c>
       <c r="C265" t="inlineStr">
         <is>
@@ -3886,7 +3886,7 @@
         <v>6</v>
       </c>
       <c r="B266" s="2" t="n">
-        <v>46019</v>
+        <v>46014</v>
       </c>
       <c r="C266" t="inlineStr">
         <is>
@@ -3899,11 +3899,11 @@
         <v>6</v>
       </c>
       <c r="B267" s="2" t="n">
-        <v>46020</v>
+        <v>46015</v>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3912,9 +3912,74 @@
         <v>6</v>
       </c>
       <c r="B268" s="2" t="n">
+        <v>46016</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>6</v>
+      </c>
+      <c r="B269" s="2" t="n">
+        <v>46017</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>6</v>
+      </c>
+      <c r="B270" s="2" t="n">
+        <v>46018</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>6</v>
+      </c>
+      <c r="B271" s="2" t="n">
+        <v>46019</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>6</v>
+      </c>
+      <c r="B272" s="2" t="n">
+        <v>46020</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>6</v>
+      </c>
+      <c r="B273" s="2" t="n">
         <v>46021</v>
       </c>
-      <c r="C268" t="inlineStr">
+      <c r="C273" t="inlineStr">
         <is>
           <t>libre</t>
         </is>

</xml_diff>

<commit_message>
Logicas DNI / Telefono / Mensajes mejores / Corpus
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C273"/>
+  <dimension ref="A1:C275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1173,33 +1173,33 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45853</v>
+        <v>46104</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45854</v>
+        <v>46105</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1208,11 +1208,11 @@
         <v>2</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45856</v>
+        <v>45853</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1221,11 +1221,11 @@
         <v>2</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45857</v>
+        <v>45854</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
         <v>2</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45884</v>
+        <v>45856</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         <v>2</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45887</v>
+        <v>45857</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
         <v>2</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45888</v>
+        <v>45884</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1273,11 +1273,11 @@
         <v>2</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45992</v>
+        <v>45887</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1286,11 +1286,11 @@
         <v>2</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45993</v>
+        <v>45888</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1299,11 +1299,11 @@
         <v>2</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45994</v>
+        <v>45992</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
         <v>2</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45995</v>
+        <v>45993</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1325,11 +1325,11 @@
         <v>2</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45996</v>
+        <v>45994</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1338,11 +1338,11 @@
         <v>2</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>45997</v>
+        <v>45995</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
         <v>2</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>45998</v>
+        <v>45996</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -1364,11 +1364,11 @@
         <v>2</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45999</v>
+        <v>45997</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>46000</v>
+        <v>45998</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -1390,11 +1390,11 @@
         <v>2</v>
       </c>
       <c r="B74" s="2" t="n">
-        <v>46001</v>
+        <v>45999</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
         <v>2</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>46002</v>
+        <v>46000</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -1416,11 +1416,11 @@
         <v>2</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>46003</v>
+        <v>46001</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
         <v>2</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>46004</v>
+        <v>46002</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -1442,7 +1442,7 @@
         <v>2</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>46005</v>
+        <v>46003</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -1455,11 +1455,11 @@
         <v>2</v>
       </c>
       <c r="B79" s="2" t="n">
-        <v>46006</v>
+        <v>46004</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
         <v>2</v>
       </c>
       <c r="B80" s="2" t="n">
-        <v>46007</v>
+        <v>46005</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -1481,7 +1481,7 @@
         <v>2</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>46008</v>
+        <v>46006</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -1494,11 +1494,11 @@
         <v>2</v>
       </c>
       <c r="B82" s="2" t="n">
-        <v>46009</v>
+        <v>46007</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1507,11 +1507,11 @@
         <v>2</v>
       </c>
       <c r="B83" s="2" t="n">
-        <v>46010</v>
+        <v>46008</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1520,11 +1520,11 @@
         <v>2</v>
       </c>
       <c r="B84" s="2" t="n">
-        <v>46011</v>
+        <v>46009</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1533,11 +1533,11 @@
         <v>2</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>46012</v>
+        <v>46010</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
         <v>2</v>
       </c>
       <c r="B86" s="2" t="n">
-        <v>46013</v>
+        <v>46011</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -1559,11 +1559,11 @@
         <v>2</v>
       </c>
       <c r="B87" s="2" t="n">
-        <v>46014</v>
+        <v>46012</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
         <v>2</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>46015</v>
+        <v>46013</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -1585,11 +1585,11 @@
         <v>2</v>
       </c>
       <c r="B89" s="2" t="n">
-        <v>46016</v>
+        <v>46014</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
         <v>2</v>
       </c>
       <c r="B90" s="2" t="n">
-        <v>46017</v>
+        <v>46015</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
         <v>2</v>
       </c>
       <c r="B91" s="2" t="n">
-        <v>46018</v>
+        <v>46016</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -1624,11 +1624,11 @@
         <v>2</v>
       </c>
       <c r="B92" s="2" t="n">
-        <v>46019</v>
+        <v>46017</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
         <v>2</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>46020</v>
+        <v>46018</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -1650,11 +1650,11 @@
         <v>2</v>
       </c>
       <c r="B94" s="2" t="n">
-        <v>46021</v>
+        <v>46019</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
         <v>2</v>
       </c>
       <c r="B95" s="2" t="n">
-        <v>46055</v>
+        <v>46020</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -1676,11 +1676,11 @@
         <v>2</v>
       </c>
       <c r="B96" s="2" t="n">
-        <v>46056</v>
+        <v>46021</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
         <v>2</v>
       </c>
       <c r="B97" s="2" t="n">
-        <v>46057</v>
+        <v>46055</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -1699,10 +1699,10 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45850</v>
+        <v>46056</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -1712,10 +1712,10 @@
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B99" s="2" t="n">
-        <v>45851</v>
+        <v>46057</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -1728,11 +1728,11 @@
         <v>3</v>
       </c>
       <c r="B100" s="2" t="n">
-        <v>45992</v>
+        <v>45850</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1741,11 +1741,11 @@
         <v>3</v>
       </c>
       <c r="B101" s="2" t="n">
-        <v>45993</v>
+        <v>45851</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1754,11 +1754,11 @@
         <v>3</v>
       </c>
       <c r="B102" s="2" t="n">
-        <v>45994</v>
+        <v>45992</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
         <v>3</v>
       </c>
       <c r="B103" s="2" t="n">
-        <v>45995</v>
+        <v>45993</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -1780,11 +1780,11 @@
         <v>3</v>
       </c>
       <c r="B104" s="2" t="n">
-        <v>45996</v>
+        <v>45994</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1793,11 +1793,11 @@
         <v>3</v>
       </c>
       <c r="B105" s="2" t="n">
-        <v>45997</v>
+        <v>45995</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
         <v>3</v>
       </c>
       <c r="B106" s="2" t="n">
-        <v>45998</v>
+        <v>45996</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -1819,11 +1819,11 @@
         <v>3</v>
       </c>
       <c r="B107" s="2" t="n">
-        <v>45999</v>
+        <v>45997</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
         <v>3</v>
       </c>
       <c r="B108" s="2" t="n">
-        <v>46000</v>
+        <v>45998</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -1845,11 +1845,11 @@
         <v>3</v>
       </c>
       <c r="B109" s="2" t="n">
-        <v>46001</v>
+        <v>45999</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
         <v>3</v>
       </c>
       <c r="B110" s="2" t="n">
-        <v>46002</v>
+        <v>46000</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -1871,11 +1871,11 @@
         <v>3</v>
       </c>
       <c r="B111" s="2" t="n">
-        <v>46003</v>
+        <v>46001</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
         <v>3</v>
       </c>
       <c r="B112" s="2" t="n">
-        <v>46004</v>
+        <v>46002</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>3</v>
       </c>
       <c r="B113" s="2" t="n">
-        <v>46005</v>
+        <v>46003</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -1910,11 +1910,11 @@
         <v>3</v>
       </c>
       <c r="B114" s="2" t="n">
-        <v>46006</v>
+        <v>46004</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
         <v>3</v>
       </c>
       <c r="B115" s="2" t="n">
-        <v>46007</v>
+        <v>46005</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -1936,11 +1936,11 @@
         <v>3</v>
       </c>
       <c r="B116" s="2" t="n">
-        <v>46008</v>
+        <v>46006</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
         <v>3</v>
       </c>
       <c r="B117" s="2" t="n">
-        <v>46009</v>
+        <v>46007</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         <v>3</v>
       </c>
       <c r="B118" s="2" t="n">
-        <v>46010</v>
+        <v>46008</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -1975,7 +1975,7 @@
         <v>3</v>
       </c>
       <c r="B119" s="2" t="n">
-        <v>46011</v>
+        <v>46009</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -1988,11 +1988,11 @@
         <v>3</v>
       </c>
       <c r="B120" s="2" t="n">
-        <v>46012</v>
+        <v>46010</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
         <v>3</v>
       </c>
       <c r="B121" s="2" t="n">
-        <v>46013</v>
+        <v>46011</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -2014,11 +2014,11 @@
         <v>3</v>
       </c>
       <c r="B122" s="2" t="n">
-        <v>46014</v>
+        <v>46012</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
         <v>3</v>
       </c>
       <c r="B123" s="2" t="n">
-        <v>46015</v>
+        <v>46013</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -2040,11 +2040,11 @@
         <v>3</v>
       </c>
       <c r="B124" s="2" t="n">
-        <v>46016</v>
+        <v>46014</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         <v>3</v>
       </c>
       <c r="B125" s="2" t="n">
-        <v>46017</v>
+        <v>46015</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
@@ -2066,11 +2066,11 @@
         <v>3</v>
       </c>
       <c r="B126" s="2" t="n">
-        <v>46018</v>
+        <v>46016</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
         <v>3</v>
       </c>
       <c r="B127" s="2" t="n">
-        <v>46019</v>
+        <v>46017</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -2092,11 +2092,11 @@
         <v>3</v>
       </c>
       <c r="B128" s="2" t="n">
-        <v>46020</v>
+        <v>46018</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
         <v>3</v>
       </c>
       <c r="B129" s="2" t="n">
-        <v>46021</v>
+        <v>46019</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -2118,11 +2118,11 @@
         <v>3</v>
       </c>
       <c r="B130" s="2" t="n">
-        <v>46068</v>
+        <v>46020</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
         <v>3</v>
       </c>
       <c r="B131" s="2" t="n">
-        <v>46069</v>
+        <v>46021</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -2144,7 +2144,7 @@
         <v>3</v>
       </c>
       <c r="B132" s="2" t="n">
-        <v>46070</v>
+        <v>46068</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
@@ -2157,7 +2157,7 @@
         <v>3</v>
       </c>
       <c r="B133" s="2" t="n">
-        <v>46071</v>
+        <v>46069</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
@@ -2170,11 +2170,11 @@
         <v>3</v>
       </c>
       <c r="B134" s="2" t="n">
-        <v>46073</v>
+        <v>46070</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2183,11 +2183,11 @@
         <v>3</v>
       </c>
       <c r="B135" s="2" t="n">
-        <v>46074</v>
+        <v>46071</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2196,7 @@
         <v>3</v>
       </c>
       <c r="B136" s="2" t="n">
-        <v>46075</v>
+        <v>46073</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
         <v>3</v>
       </c>
       <c r="B137" s="2" t="n">
-        <v>46077</v>
+        <v>46074</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
         <v>3</v>
       </c>
       <c r="B138" s="2" t="n">
-        <v>46078</v>
+        <v>46075</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
         <v>3</v>
       </c>
       <c r="B139" s="2" t="n">
-        <v>46079</v>
+        <v>46077</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         <v>3</v>
       </c>
       <c r="B140" s="2" t="n">
-        <v>46080</v>
+        <v>46078</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         <v>3</v>
       </c>
       <c r="B141" s="2" t="n">
-        <v>46103</v>
+        <v>46079</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         <v>3</v>
       </c>
       <c r="B142" s="2" t="n">
-        <v>46104</v>
+        <v>46080</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v>3</v>
       </c>
       <c r="B143" s="2" t="n">
-        <v>46105</v>
+        <v>46103</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v>3</v>
       </c>
       <c r="B144" s="2" t="n">
-        <v>46106</v>
+        <v>46104</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         <v>3</v>
       </c>
       <c r="B145" s="2" t="n">
-        <v>46108</v>
+        <v>46105</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         <v>3</v>
       </c>
       <c r="B146" s="2" t="n">
-        <v>46109</v>
+        <v>46106</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
@@ -2339,7 +2339,7 @@
         <v>3</v>
       </c>
       <c r="B147" s="2" t="n">
-        <v>46392</v>
+        <v>46108</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -2352,7 +2352,7 @@
         <v>3</v>
       </c>
       <c r="B148" s="2" t="n">
-        <v>46393</v>
+        <v>46109</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         <v>3</v>
       </c>
       <c r="B149" s="2" t="n">
-        <v>46394</v>
+        <v>46392</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
@@ -2378,7 +2378,7 @@
         <v>3</v>
       </c>
       <c r="B150" s="2" t="n">
-        <v>46395</v>
+        <v>46393</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
@@ -2391,7 +2391,7 @@
         <v>3</v>
       </c>
       <c r="B151" s="2" t="n">
-        <v>46396</v>
+        <v>46394</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
@@ -2401,27 +2401,27 @@
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B152" s="2" t="n">
-        <v>45658</v>
+        <v>46395</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B153" s="2" t="n">
-        <v>45659</v>
+        <v>46396</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2430,7 @@
         <v>4</v>
       </c>
       <c r="B154" s="2" t="n">
-        <v>45660</v>
+        <v>45658</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -2443,7 +2443,7 @@
         <v>4</v>
       </c>
       <c r="B155" s="2" t="n">
-        <v>45661</v>
+        <v>45659</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
         <v>4</v>
       </c>
       <c r="B156" s="2" t="n">
-        <v>45992</v>
+        <v>45660</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         <v>4</v>
       </c>
       <c r="B157" s="2" t="n">
-        <v>45993</v>
+        <v>45661</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
@@ -2482,11 +2482,11 @@
         <v>4</v>
       </c>
       <c r="B158" s="2" t="n">
-        <v>45994</v>
+        <v>45992</v>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2495,7 @@
         <v>4</v>
       </c>
       <c r="B159" s="2" t="n">
-        <v>45995</v>
+        <v>45993</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -2508,11 +2508,11 @@
         <v>4</v>
       </c>
       <c r="B160" s="2" t="n">
-        <v>45996</v>
+        <v>45994</v>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2521,11 +2521,11 @@
         <v>4</v>
       </c>
       <c r="B161" s="2" t="n">
-        <v>45997</v>
+        <v>45995</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
         <v>4</v>
       </c>
       <c r="B162" s="2" t="n">
-        <v>45998</v>
+        <v>45996</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -2547,11 +2547,11 @@
         <v>4</v>
       </c>
       <c r="B163" s="2" t="n">
-        <v>45999</v>
+        <v>45997</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2560,7 @@
         <v>4</v>
       </c>
       <c r="B164" s="2" t="n">
-        <v>46000</v>
+        <v>45998</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
@@ -2573,11 +2573,11 @@
         <v>4</v>
       </c>
       <c r="B165" s="2" t="n">
-        <v>46001</v>
+        <v>45999</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
         <v>4</v>
       </c>
       <c r="B166" s="2" t="n">
-        <v>46002</v>
+        <v>46000</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -2599,11 +2599,11 @@
         <v>4</v>
       </c>
       <c r="B167" s="2" t="n">
-        <v>46003</v>
+        <v>46001</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>4</v>
       </c>
       <c r="B168" s="2" t="n">
-        <v>46004</v>
+        <v>46002</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
         <v>4</v>
       </c>
       <c r="B169" s="2" t="n">
-        <v>46005</v>
+        <v>46003</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -2638,11 +2638,11 @@
         <v>4</v>
       </c>
       <c r="B170" s="2" t="n">
-        <v>46006</v>
+        <v>46004</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
         <v>4</v>
       </c>
       <c r="B171" s="2" t="n">
-        <v>46007</v>
+        <v>46005</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
@@ -2664,11 +2664,11 @@
         <v>4</v>
       </c>
       <c r="B172" s="2" t="n">
-        <v>46008</v>
+        <v>46006</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
         <v>4</v>
       </c>
       <c r="B173" s="2" t="n">
-        <v>46009</v>
+        <v>46007</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
@@ -2690,7 +2690,7 @@
         <v>4</v>
       </c>
       <c r="B174" s="2" t="n">
-        <v>46010</v>
+        <v>46008</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
@@ -2703,7 +2703,7 @@
         <v>4</v>
       </c>
       <c r="B175" s="2" t="n">
-        <v>46011</v>
+        <v>46009</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
@@ -2716,11 +2716,11 @@
         <v>4</v>
       </c>
       <c r="B176" s="2" t="n">
-        <v>46012</v>
+        <v>46010</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>4</v>
       </c>
       <c r="B177" s="2" t="n">
-        <v>46013</v>
+        <v>46011</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
@@ -2742,11 +2742,11 @@
         <v>4</v>
       </c>
       <c r="B178" s="2" t="n">
-        <v>46014</v>
+        <v>46012</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
         <v>4</v>
       </c>
       <c r="B179" s="2" t="n">
-        <v>46015</v>
+        <v>46013</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
@@ -2768,11 +2768,11 @@
         <v>4</v>
       </c>
       <c r="B180" s="2" t="n">
-        <v>46016</v>
+        <v>46014</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
         <v>4</v>
       </c>
       <c r="B181" s="2" t="n">
-        <v>46017</v>
+        <v>46015</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
@@ -2794,11 +2794,11 @@
         <v>4</v>
       </c>
       <c r="B182" s="2" t="n">
-        <v>46018</v>
+        <v>46016</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
         <v>4</v>
       </c>
       <c r="B183" s="2" t="n">
-        <v>46019</v>
+        <v>46017</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -2820,11 +2820,11 @@
         <v>4</v>
       </c>
       <c r="B184" s="2" t="n">
-        <v>46020</v>
+        <v>46018</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
         <v>4</v>
       </c>
       <c r="B185" s="2" t="n">
-        <v>46021</v>
+        <v>46019</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -2846,11 +2846,11 @@
         <v>4</v>
       </c>
       <c r="B186" s="2" t="n">
-        <v>46023</v>
+        <v>46020</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
         <v>4</v>
       </c>
       <c r="B187" s="2" t="n">
-        <v>46024</v>
+        <v>46021</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
         <v>4</v>
       </c>
       <c r="B188" s="2" t="n">
-        <v>46025</v>
+        <v>46023</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
@@ -2885,7 +2885,7 @@
         <v>4</v>
       </c>
       <c r="B189" s="2" t="n">
-        <v>46026</v>
+        <v>46024</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
         <v>4</v>
       </c>
       <c r="B190" s="2" t="n">
-        <v>46027</v>
+        <v>46025</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -2911,7 +2911,7 @@
         <v>4</v>
       </c>
       <c r="B191" s="2" t="n">
-        <v>46028</v>
+        <v>46026</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -2924,7 +2924,7 @@
         <v>4</v>
       </c>
       <c r="B192" s="2" t="n">
-        <v>46038</v>
+        <v>46027</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
         <v>4</v>
       </c>
       <c r="B193" s="2" t="n">
-        <v>46039</v>
+        <v>46028</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -2950,7 +2950,7 @@
         <v>4</v>
       </c>
       <c r="B194" s="2" t="n">
-        <v>46042</v>
+        <v>46038</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
@@ -2963,7 +2963,7 @@
         <v>4</v>
       </c>
       <c r="B195" s="2" t="n">
-        <v>46043</v>
+        <v>46039</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v>4</v>
       </c>
       <c r="B196" s="2" t="n">
-        <v>46044</v>
+        <v>46042</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
         <v>4</v>
       </c>
       <c r="B197" s="2" t="n">
-        <v>46063</v>
+        <v>46043</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
         <v>4</v>
       </c>
       <c r="B198" s="2" t="n">
-        <v>46064</v>
+        <v>46044</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
@@ -3015,11 +3015,11 @@
         <v>4</v>
       </c>
       <c r="B199" s="2" t="n">
-        <v>46078</v>
+        <v>46063</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3028,37 +3028,37 @@
         <v>4</v>
       </c>
       <c r="B200" s="2" t="n">
-        <v>46079</v>
+        <v>46064</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B201" s="2" t="n">
-        <v>45992</v>
+        <v>46078</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B202" s="2" t="n">
-        <v>45993</v>
+        <v>46079</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3067,11 +3067,11 @@
         <v>5</v>
       </c>
       <c r="B203" s="2" t="n">
-        <v>45994</v>
+        <v>45992</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
         <v>5</v>
       </c>
       <c r="B204" s="2" t="n">
-        <v>45995</v>
+        <v>45993</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
@@ -3093,11 +3093,11 @@
         <v>5</v>
       </c>
       <c r="B205" s="2" t="n">
-        <v>45996</v>
+        <v>45994</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3106,11 +3106,11 @@
         <v>5</v>
       </c>
       <c r="B206" s="2" t="n">
-        <v>45997</v>
+        <v>45995</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
         <v>5</v>
       </c>
       <c r="B207" s="2" t="n">
-        <v>45998</v>
+        <v>45996</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
@@ -3132,11 +3132,11 @@
         <v>5</v>
       </c>
       <c r="B208" s="2" t="n">
-        <v>45999</v>
+        <v>45997</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
         <v>5</v>
       </c>
       <c r="B209" s="2" t="n">
-        <v>46000</v>
+        <v>45998</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -3158,11 +3158,11 @@
         <v>5</v>
       </c>
       <c r="B210" s="2" t="n">
-        <v>46001</v>
+        <v>45999</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
         <v>5</v>
       </c>
       <c r="B211" s="2" t="n">
-        <v>46002</v>
+        <v>46000</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
@@ -3184,7 +3184,7 @@
         <v>5</v>
       </c>
       <c r="B212" s="2" t="n">
-        <v>46003</v>
+        <v>46001</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
@@ -3197,11 +3197,11 @@
         <v>5</v>
       </c>
       <c r="B213" s="2" t="n">
-        <v>46004</v>
+        <v>46002</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3210,11 +3210,11 @@
         <v>5</v>
       </c>
       <c r="B214" s="2" t="n">
-        <v>46005</v>
+        <v>46003</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
         <v>5</v>
       </c>
       <c r="B215" s="2" t="n">
-        <v>46006</v>
+        <v>46004</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         <v>5</v>
       </c>
       <c r="B216" s="2" t="n">
-        <v>46007</v>
+        <v>46005</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
@@ -3249,11 +3249,11 @@
         <v>5</v>
       </c>
       <c r="B217" s="2" t="n">
-        <v>46008</v>
+        <v>46006</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
         <v>5</v>
       </c>
       <c r="B218" s="2" t="n">
-        <v>46009</v>
+        <v>46007</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
@@ -3275,7 +3275,7 @@
         <v>5</v>
       </c>
       <c r="B219" s="2" t="n">
-        <v>46010</v>
+        <v>46008</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
         <v>5</v>
       </c>
       <c r="B220" s="2" t="n">
-        <v>46011</v>
+        <v>46009</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
@@ -3301,11 +3301,11 @@
         <v>5</v>
       </c>
       <c r="B221" s="2" t="n">
-        <v>46012</v>
+        <v>46010</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
         <v>5</v>
       </c>
       <c r="B222" s="2" t="n">
-        <v>46013</v>
+        <v>46011</v>
       </c>
       <c r="C222" t="inlineStr">
         <is>
@@ -3327,11 +3327,11 @@
         <v>5</v>
       </c>
       <c r="B223" s="2" t="n">
-        <v>46014</v>
+        <v>46012</v>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
         <v>5</v>
       </c>
       <c r="B224" s="2" t="n">
-        <v>46015</v>
+        <v>46013</v>
       </c>
       <c r="C224" t="inlineStr">
         <is>
@@ -3353,11 +3353,11 @@
         <v>5</v>
       </c>
       <c r="B225" s="2" t="n">
-        <v>46016</v>
+        <v>46014</v>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
         <v>5</v>
       </c>
       <c r="B226" s="2" t="n">
-        <v>46017</v>
+        <v>46015</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
@@ -3379,11 +3379,11 @@
         <v>5</v>
       </c>
       <c r="B227" s="2" t="n">
-        <v>46018</v>
+        <v>46016</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
         <v>5</v>
       </c>
       <c r="B228" s="2" t="n">
-        <v>46019</v>
+        <v>46017</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
@@ -3405,11 +3405,11 @@
         <v>5</v>
       </c>
       <c r="B229" s="2" t="n">
-        <v>46020</v>
+        <v>46018</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
         <v>5</v>
       </c>
       <c r="B230" s="2" t="n">
-        <v>46021</v>
+        <v>46019</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
@@ -3428,10 +3428,10 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B231" s="2" t="n">
-        <v>45850</v>
+        <v>46020</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
@@ -3441,14 +3441,14 @@
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B232" s="2" t="n">
-        <v>45851</v>
+        <v>46021</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
         <v>6</v>
       </c>
       <c r="B233" s="2" t="n">
-        <v>45860</v>
+        <v>45850</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
@@ -3470,7 +3470,7 @@
         <v>6</v>
       </c>
       <c r="B234" s="2" t="n">
-        <v>45861</v>
+        <v>45851</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         <v>6</v>
       </c>
       <c r="B235" s="2" t="n">
-        <v>45862</v>
+        <v>45860</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
@@ -3496,7 +3496,7 @@
         <v>6</v>
       </c>
       <c r="B236" s="2" t="n">
-        <v>45863</v>
+        <v>45861</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -3509,11 +3509,11 @@
         <v>6</v>
       </c>
       <c r="B237" s="2" t="n">
-        <v>45867</v>
+        <v>45862</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3522,11 +3522,11 @@
         <v>6</v>
       </c>
       <c r="B238" s="2" t="n">
-        <v>45868</v>
+        <v>45863</v>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3535,7 @@
         <v>6</v>
       </c>
       <c r="B239" s="2" t="n">
-        <v>45869</v>
+        <v>45867</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
         <v>6</v>
       </c>
       <c r="B240" s="2" t="n">
-        <v>45870</v>
+        <v>45868</v>
       </c>
       <c r="C240" t="inlineStr">
         <is>
@@ -3561,11 +3561,11 @@
         <v>6</v>
       </c>
       <c r="B241" s="2" t="n">
-        <v>45884</v>
+        <v>45869</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3574,11 +3574,11 @@
         <v>6</v>
       </c>
       <c r="B242" s="2" t="n">
-        <v>45885</v>
+        <v>45870</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3587,7 +3587,7 @@
         <v>6</v>
       </c>
       <c r="B243" s="2" t="n">
-        <v>45886</v>
+        <v>45884</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
@@ -3600,11 +3600,11 @@
         <v>6</v>
       </c>
       <c r="B244" s="2" t="n">
-        <v>45992</v>
+        <v>45885</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3613,11 +3613,11 @@
         <v>6</v>
       </c>
       <c r="B245" s="2" t="n">
-        <v>45993</v>
+        <v>45886</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3626,11 +3626,11 @@
         <v>6</v>
       </c>
       <c r="B246" s="2" t="n">
-        <v>45994</v>
+        <v>45992</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
         <v>6</v>
       </c>
       <c r="B247" s="2" t="n">
-        <v>45995</v>
+        <v>45993</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -3652,11 +3652,11 @@
         <v>6</v>
       </c>
       <c r="B248" s="2" t="n">
-        <v>45996</v>
+        <v>45994</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3665,11 +3665,11 @@
         <v>6</v>
       </c>
       <c r="B249" s="2" t="n">
-        <v>45997</v>
+        <v>45995</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3678,7 @@
         <v>6</v>
       </c>
       <c r="B250" s="2" t="n">
-        <v>45998</v>
+        <v>45996</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -3691,11 +3691,11 @@
         <v>6</v>
       </c>
       <c r="B251" s="2" t="n">
-        <v>45999</v>
+        <v>45997</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3704,7 @@
         <v>6</v>
       </c>
       <c r="B252" s="2" t="n">
-        <v>46000</v>
+        <v>45998</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -3717,11 +3717,11 @@
         <v>6</v>
       </c>
       <c r="B253" s="2" t="n">
-        <v>46001</v>
+        <v>45999</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3730,7 +3730,7 @@
         <v>6</v>
       </c>
       <c r="B254" s="2" t="n">
-        <v>46002</v>
+        <v>46000</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
@@ -3743,11 +3743,11 @@
         <v>6</v>
       </c>
       <c r="B255" s="2" t="n">
-        <v>46003</v>
+        <v>46001</v>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3756,7 +3756,7 @@
         <v>6</v>
       </c>
       <c r="B256" s="2" t="n">
-        <v>46004</v>
+        <v>46002</v>
       </c>
       <c r="C256" t="inlineStr">
         <is>
@@ -3769,7 +3769,7 @@
         <v>6</v>
       </c>
       <c r="B257" s="2" t="n">
-        <v>46005</v>
+        <v>46003</v>
       </c>
       <c r="C257" t="inlineStr">
         <is>
@@ -3782,11 +3782,11 @@
         <v>6</v>
       </c>
       <c r="B258" s="2" t="n">
-        <v>46006</v>
+        <v>46004</v>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
         <v>6</v>
       </c>
       <c r="B259" s="2" t="n">
-        <v>46007</v>
+        <v>46005</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
@@ -3808,11 +3808,11 @@
         <v>6</v>
       </c>
       <c r="B260" s="2" t="n">
-        <v>46008</v>
+        <v>46006</v>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
         <v>6</v>
       </c>
       <c r="B261" s="2" t="n">
-        <v>46009</v>
+        <v>46007</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
@@ -3834,7 +3834,7 @@
         <v>6</v>
       </c>
       <c r="B262" s="2" t="n">
-        <v>46010</v>
+        <v>46008</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
@@ -3847,7 +3847,7 @@
         <v>6</v>
       </c>
       <c r="B263" s="2" t="n">
-        <v>46011</v>
+        <v>46009</v>
       </c>
       <c r="C263" t="inlineStr">
         <is>
@@ -3860,11 +3860,11 @@
         <v>6</v>
       </c>
       <c r="B264" s="2" t="n">
-        <v>46012</v>
+        <v>46010</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3873,7 +3873,7 @@
         <v>6</v>
       </c>
       <c r="B265" s="2" t="n">
-        <v>46013</v>
+        <v>46011</v>
       </c>
       <c r="C265" t="inlineStr">
         <is>
@@ -3886,11 +3886,11 @@
         <v>6</v>
       </c>
       <c r="B266" s="2" t="n">
-        <v>46014</v>
+        <v>46012</v>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
         <v>6</v>
       </c>
       <c r="B267" s="2" t="n">
-        <v>46015</v>
+        <v>46013</v>
       </c>
       <c r="C267" t="inlineStr">
         <is>
@@ -3912,11 +3912,11 @@
         <v>6</v>
       </c>
       <c r="B268" s="2" t="n">
-        <v>46016</v>
+        <v>46014</v>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
         <v>6</v>
       </c>
       <c r="B269" s="2" t="n">
-        <v>46017</v>
+        <v>46015</v>
       </c>
       <c r="C269" t="inlineStr">
         <is>
@@ -3938,11 +3938,11 @@
         <v>6</v>
       </c>
       <c r="B270" s="2" t="n">
-        <v>46018</v>
+        <v>46016</v>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>ocupado</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
         <v>6</v>
       </c>
       <c r="B271" s="2" t="n">
-        <v>46019</v>
+        <v>46017</v>
       </c>
       <c r="C271" t="inlineStr">
         <is>
@@ -3964,11 +3964,11 @@
         <v>6</v>
       </c>
       <c r="B272" s="2" t="n">
-        <v>46020</v>
+        <v>46018</v>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ocupado</t>
+          <t>libre</t>
         </is>
       </c>
     </row>
@@ -3977,9 +3977,35 @@
         <v>6</v>
       </c>
       <c r="B273" s="2" t="n">
+        <v>46019</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>6</v>
+      </c>
+      <c r="B274" s="2" t="n">
+        <v>46020</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>ocupado</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>6</v>
+      </c>
+      <c r="B275" s="2" t="n">
         <v>46021</v>
       </c>
-      <c r="C273" t="inlineStr">
+      <c r="C275" t="inlineStr">
         <is>
           <t>libre</t>
         </is>

</xml_diff>